<commit_message>
CoreWeave quarterly history from earnings releases; disclosed-KPI dataset
Operating KPIs that SEC's structured data does not carry (active power,
contracted power, revenue backlog, adjusted EBITDA) are read from the press
releases attached to each quarter's 8-K into data/disclosed/CRWV.csv, one
row per figure with its source; every row was checked against the sentence
that states it. The EDGAR client can now list and download filing exhibits.

CoreWeave v1 is a six-quarter history, per MW of average active power (no
assumptions) and per installed GPU-hour (one assumption: kW per GPU). Excel
formulas are re-evaluated against the Python values for every column.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models/CRWV.xlsx
+++ b/models/CRWV.xlsx
@@ -36,9 +36,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0.00##"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -55,10 +56,13 @@
       <color rgb="000000FF"/>
     </font>
     <font>
-      <color rgb="00008000"/>
+      <color rgb="00595959"/>
     </font>
     <font>
       <color rgb="00000000"/>
+    </font>
+    <font>
+      <color rgb="00008000"/>
     </font>
     <font>
       <b val="1"/>
@@ -66,9 +70,6 @@
     </font>
     <font>
       <i val="1"/>
-    </font>
-    <font>
-      <color rgb="00595959"/>
     </font>
     <font>
       <i val="1"/>
@@ -100,18 +101,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,7 +122,11 @@
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -747,7 +752,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>[derived; proposed] Technology equipment, gross 9,146,575 thousand divided by more than 250,000 GPUs at Dec 31, 2024. A fleet average that includes servers and networking and excludes construction in progress. Newer GPU generations cost more than this average.</t>
+          <t>[derived; proposed] Technology equipment, gross 9,146,575 thousand divided by more than 250,000 GPUs at Dec 31, 2024. A fleet average that includes servers and networking and excludes construction in progress. Compare with the model's capex per MW added (Outputs sheet), which is the same idea measured from cash flows.</t>
         </is>
       </c>
     </row>
@@ -772,7 +777,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>[derived; proposed] More than 360 MW of active power divided by more than 250,000 GPUs at Dec 31, 2024. Facility-level power per GPU, so cooling and non-GPU load are already inside it.</t>
+          <t>[derived; proposed] More than 360 MW of active power divided by more than 250,000 GPUs at Dec 31, 2024. Facility-level power per GPU, so cooling and non-GPU load are already inside it. This is the ONE assumption that converts disclosed MW into GPU counts; every per-GPU line scales with it, the per-MW lines do not use it.</t>
         </is>
       </c>
     </row>
@@ -835,7 +840,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>[judgment; proposed] Set to 1.0 because price_per_gpu_hour below is revenue per INSTALLED hour. Idle and not-yet-billing GPUs are already inside that price.</t>
+          <t>[judgment; proposed] Set to 1.0 because the model measures revenue per INSTALLED GPU-hour (quarterly revenue over average installed capacity). Idle and not-yet-billing GPUs are already inside that figure. Only used by the per-GPU lines.</t>
         </is>
       </c>
     </row>
@@ -938,21 +943,17 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1.354</v>
+        <v>0</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>USD/GPU-hour</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>S-1 p.113, p.2</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>[derived; proposed] Q4 2024 revenue 747,430 thousand divided by 250,000 GPUs times 2,208 hours. Realised revenue per installed GPU-hour across the whole fleet. It is NOT a contract price, and it is understated because the year-end GPU count is applied to the whole quarter.</t>
+          <t>[judgment; proposed] Not used: the model computes revenue per installed GPU-hour for each quarter from reported revenue and disclosed capacity (see the Outputs sheet). Kept at 0 so the engine's rental mode has a defined input.</t>
         </is>
       </c>
     </row>
@@ -984,21 +985,17 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>0.4734</v>
+        <v>0</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>USD/GPU-hour</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>S-1 p.113, p.115, p.2</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>[derived; proposed] Q4 2024 revenue less adjusted EBITDA (747,430 less 486,114 thousand) per installed GPU-hour. Lumps energy, data-centre leases, staff and everything else above adjusted EBITDA into one number.</t>
+          <t>[judgment; proposed] Not used: each quarter's cash cost per GPU-hour is revenue less adjusted EBITDA over installed GPU-hours, computed by the model. Kept at 0.</t>
         </is>
       </c>
     </row>
@@ -1080,12 +1077,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1101,135 +1103,490 @@
       </c>
       <c r="C1" s="13" t="inlineStr">
         <is>
-          <t>2024Q4</t>
+          <t>2025Q1</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>2025Q2</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>2025Q3</t>
+        </is>
+      </c>
+      <c r="F1" s="13" t="inlineStr">
+        <is>
+          <t>2025Q4</t>
+        </is>
+      </c>
+      <c r="G1" s="13" t="inlineStr">
+        <is>
+          <t>2026Q1</t>
+        </is>
+      </c>
+      <c r="H1" s="13" t="inlineStr">
+        <is>
+          <t>2026Q2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Active power, end of quarter</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="n">
+        <v>420</v>
+      </c>
+      <c r="D2" s="14" t="n">
+        <v>470</v>
+      </c>
+      <c r="E2" s="14" t="n">
+        <v>590</v>
+      </c>
+      <c r="F2" s="14" t="n">
+        <v>850</v>
+      </c>
+      <c r="G2" s="14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H2" s="14" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Active power added</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D3" s="15">
+        <f>D2-C2</f>
+        <v/>
+      </c>
+      <c r="E3" s="15">
+        <f>E2-D2</f>
+        <v/>
+      </c>
+      <c r="F3" s="15">
+        <f>F2-E2</f>
+        <v/>
+      </c>
+      <c r="G3" s="15">
+        <f>G2-F2</f>
+        <v/>
+      </c>
+      <c r="H3" s="15">
+        <f>H2-G2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Active power, average</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>390</v>
+      </c>
+      <c r="D4" s="15">
+        <f>(C2+D2)/2</f>
+        <v/>
+      </c>
+      <c r="E4" s="15">
+        <f>(D2+E2)/2</f>
+        <v/>
+      </c>
+      <c r="F4" s="15">
+        <f>(E2+F2)/2</f>
+        <v/>
+      </c>
+      <c r="G4" s="15">
+        <f>(F2+G2)/2</f>
+        <v/>
+      </c>
+      <c r="H4" s="15">
+        <f>(G2+H2)/2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Contracted power</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GW</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Revenue backlog</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>USD bn</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Hours in the quarter</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>2160</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>2184</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>2208</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>2208</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>2160</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>2184</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GPUs installed, average (from MW and kW per GPU)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GPUs</t>
+        </is>
+      </c>
+      <c r="C8" s="17">
+        <f>C4*1000/in_power_draw_kw</f>
+        <v/>
+      </c>
+      <c r="D8" s="17">
+        <f>D4*1000/in_power_draw_kw</f>
+        <v/>
+      </c>
+      <c r="E8" s="17">
+        <f>E4*1000/in_power_draw_kw</f>
+        <v/>
+      </c>
+      <c r="F8" s="17">
+        <f>F4*1000/in_power_draw_kw</f>
+        <v/>
+      </c>
+      <c r="G8" s="17">
+        <f>G4*1000/in_power_draw_kw</f>
+        <v/>
+      </c>
+      <c r="H8" s="17">
+        <f>H4*1000/in_power_draw_kw</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Installed GPU-hours</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>millions</t>
+        </is>
+      </c>
+      <c r="C9" s="15">
+        <f>C8*C7/1000000</f>
+        <v/>
+      </c>
+      <c r="D9" s="15">
+        <f>D8*D7/1000000</f>
+        <v/>
+      </c>
+      <c r="E9" s="15">
+        <f>E8*E7/1000000</f>
+        <v/>
+      </c>
+      <c r="F9" s="15">
+        <f>F8*F7/1000000</f>
+        <v/>
+      </c>
+      <c r="G9" s="15">
+        <f>G8*G7/1000000</f>
+        <v/>
+      </c>
+      <c r="H9" s="15">
+        <f>H8*H7/1000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>982</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>1212</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>1364.676</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>1571.904</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>2078</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>2575</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Adjusted EBITDA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>606.131</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>753.169</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>838.124</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>898</v>
+      </c>
+      <c r="G11" s="16" t="n">
+        <v>1157</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Capital expenditure</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>1407</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>2453</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>2389.239</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>4059.761</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>7695</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <v>6422</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Capital expenditure, cumulative</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>1407</v>
+      </c>
+      <c r="D13" s="18">
+        <f>C13+D12</f>
+        <v/>
+      </c>
+      <c r="E13" s="18">
+        <f>D13+E12</f>
+        <v/>
+      </c>
+      <c r="F13" s="18">
+        <f>E13+F12</f>
+        <v/>
+      </c>
+      <c r="G13" s="18">
+        <f>F13+G12</f>
+        <v/>
+      </c>
+      <c r="H13" s="18">
+        <f>G13+H12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Active power added, cumulative</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MW</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="D14" s="15">
+        <f>C14+D3</f>
+        <v/>
+      </c>
+      <c r="E14" s="15">
+        <f>D14+E3</f>
+        <v/>
+      </c>
+      <c r="F14" s="15">
+        <f>E14+F3</f>
+        <v/>
+      </c>
+      <c r="G14" s="15">
+        <f>F14+G3</f>
+        <v/>
+      </c>
+      <c r="H14" s="15">
+        <f>G14+H3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>Capital recovery factor (share of price due each year)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>ratio</t>
         </is>
       </c>
-      <c r="C2" s="14">
+      <c r="C15" s="17">
         <f>IF(in_financing_rate=0,1/in_depreciation_years,in_financing_rate/(1-(1+in_financing_rate)^-in_depreciation_years))</f>
         <v/>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Capital charge</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>USD/GPU-hour</t>
-        </is>
-      </c>
-      <c r="C3" s="14">
-        <f>in_chip_cost*(1-in_residual_value_share/(1+in_financing_rate)^in_depreciation_years)*C2/8760</f>
+      <c r="D15" s="17">
+        <f>IF(in_financing_rate=0,1/in_depreciation_years,in_financing_rate/(1-(1+in_financing_rate)^-in_depreciation_years))</f>
         <v/>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>USD/GPU-hour</t>
-        </is>
-      </c>
-      <c r="C4" s="14">
-        <f>in_power_draw_kw*in_pue*in_electricity_price_kwh*(in_utilization+(1-in_utilization)*in_idle_power_share)</f>
+      <c r="E15" s="17">
+        <f>IF(in_financing_rate=0,1/in_depreciation_years,in_financing_rate/(1-(1+in_financing_rate)^-in_depreciation_years))</f>
         <v/>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Data-centre space</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>USD/GPU-hour</t>
-        </is>
-      </c>
-      <c r="C5" s="14">
-        <f>in_facility_cost_per_kw_month*in_power_draw_kw*12/8760</f>
+      <c r="F15" s="17">
+        <f>IF(in_financing_rate=0,1/in_depreciation_years,in_financing_rate/(1-(1+in_financing_rate)^-in_depreciation_years))</f>
         <v/>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Other operating cost</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>USD/GPU-hour</t>
-        </is>
-      </c>
-      <c r="C6" s="14">
-        <f>in_other_opex_per_gpu_hour</f>
+      <c r="G15" s="17">
+        <f>IF(in_financing_rate=0,1/in_depreciation_years,in_financing_rate/(1-(1+in_financing_rate)^-in_depreciation_years))</f>
         <v/>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Cash cost</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>USD/GPU-hour</t>
-        </is>
-      </c>
-      <c r="C7" s="15">
-        <f>C4+C5+C6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Fully loaded cost</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>USD/GPU-hour</t>
-        </is>
-      </c>
-      <c r="C8" s="15">
-        <f>C7+C3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>USD/GPU-hour</t>
-        </is>
-      </c>
-      <c r="C9" s="14">
-        <f>in_price_per_gpu_hour*in_utilization</f>
+      <c r="H15" s="17">
+        <f>IF(in_financing_rate=0,1/in_depreciation_years,in_financing_rate/(1-(1+in_financing_rate)^-in_depreciation_years))</f>
         <v/>
       </c>
     </row>
@@ -1244,12 +1601,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1265,78 +1627,183 @@
       </c>
       <c r="C1" s="13" t="inlineStr">
         <is>
-          <t>2024Q4</t>
+          <t>2025Q1</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>2025Q2</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>2025Q3</t>
+        </is>
+      </c>
+      <c r="F1" s="13" t="inlineStr">
+        <is>
+          <t>2025Q4</t>
+        </is>
+      </c>
+      <c r="G1" s="13" t="inlineStr">
+        <is>
+          <t>2026Q1</t>
+        </is>
+      </c>
+      <c r="H1" s="13" t="inlineStr">
+        <is>
+          <t>2026Q2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cash margin</t>
+          <t>Revenue per MW, annualised</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>USD/GPU-hour</t>
-        </is>
-      </c>
-      <c r="C2" s="14">
-        <f>Drivers!C9-Drivers!C7</f>
+          <t>USD m</t>
+        </is>
+      </c>
+      <c r="C2" s="19">
+        <f>Drivers!C10*4/Drivers!C4</f>
+        <v/>
+      </c>
+      <c r="D2" s="19">
+        <f>Drivers!D10*4/Drivers!D4</f>
+        <v/>
+      </c>
+      <c r="E2" s="19">
+        <f>Drivers!E10*4/Drivers!E4</f>
+        <v/>
+      </c>
+      <c r="F2" s="19">
+        <f>Drivers!F10*4/Drivers!F4</f>
+        <v/>
+      </c>
+      <c r="G2" s="19">
+        <f>Drivers!G10*4/Drivers!G4</f>
+        <v/>
+      </c>
+      <c r="H2" s="19">
+        <f>Drivers!H10*4/Drivers!H4</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cash margin, share of revenue</t>
+          <t>Adjusted EBITDA per MW, annualised</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="C3" s="16">
-        <f>C2/Drivers!C9</f>
+          <t>USD m</t>
+        </is>
+      </c>
+      <c r="C3" s="19">
+        <f>Drivers!C11*4/Drivers!C4</f>
+        <v/>
+      </c>
+      <c r="D3" s="19">
+        <f>Drivers!D11*4/Drivers!D4</f>
+        <v/>
+      </c>
+      <c r="E3" s="19">
+        <f>Drivers!E11*4/Drivers!E4</f>
+        <v/>
+      </c>
+      <c r="F3" s="19">
+        <f>Drivers!F11*4/Drivers!F4</f>
+        <v/>
+      </c>
+      <c r="G3" s="19">
+        <f>Drivers!G11*4/Drivers!G4</f>
+        <v/>
+      </c>
+      <c r="H3" s="19">
+        <f>Drivers!H11*4/Drivers!H4</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fully loaded margin</t>
+          <t>Adjusted EBITDA margin</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>USD/GPU-hour</t>
-        </is>
-      </c>
-      <c r="C4" s="14">
-        <f>Drivers!C9-Drivers!C8</f>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C4" s="20">
+        <f>Drivers!C11/Drivers!C10</f>
+        <v/>
+      </c>
+      <c r="D4" s="20">
+        <f>Drivers!D11/Drivers!D10</f>
+        <v/>
+      </c>
+      <c r="E4" s="20">
+        <f>Drivers!E11/Drivers!E10</f>
+        <v/>
+      </c>
+      <c r="F4" s="20">
+        <f>Drivers!F11/Drivers!F10</f>
+        <v/>
+      </c>
+      <c r="G4" s="20">
+        <f>Drivers!G11/Drivers!G10</f>
+        <v/>
+      </c>
+      <c r="H4" s="20">
+        <f>Drivers!H11/Drivers!H10</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Break-even rental price</t>
+          <t>Capex per MW added, cumulative since the first quarter</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>USD/GPU-hour</t>
-        </is>
-      </c>
-      <c r="C5" s="14">
-        <f>Drivers!C8/in_utilization</f>
+          <t>USD m</t>
+        </is>
+      </c>
+      <c r="C5" s="19">
+        <f>Drivers!C13/Drivers!C14</f>
+        <v/>
+      </c>
+      <c r="D5" s="19">
+        <f>Drivers!D13/Drivers!D14</f>
+        <v/>
+      </c>
+      <c r="E5" s="19">
+        <f>Drivers!E13/Drivers!E14</f>
+        <v/>
+      </c>
+      <c r="F5" s="19">
+        <f>Drivers!F13/Drivers!F14</f>
+        <v/>
+      </c>
+      <c r="G5" s="19">
+        <f>Drivers!G13/Drivers!G14</f>
+        <v/>
+      </c>
+      <c r="H5" s="19">
+        <f>Drivers!H13/Drivers!H14</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Payback, model</t>
+          <t>Payback per MW: capex per MW / EBITDA per MW</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1344,40 +1811,316 @@
           <t>years</t>
         </is>
       </c>
-      <c r="C6" s="14">
-        <f>IF(C2&gt;0,in_chip_cost/(C2*8760),"never")</f>
+      <c r="C6" s="15">
+        <f>C5/C3</f>
+        <v/>
+      </c>
+      <c r="D6" s="15">
+        <f>D5/D3</f>
+        <v/>
+      </c>
+      <c r="E6" s="15">
+        <f>E5/E3</f>
+        <v/>
+      </c>
+      <c r="F6" s="15">
+        <f>F5/F3</f>
+        <v/>
+      </c>
+      <c r="G6" s="15">
+        <f>G5/G3</f>
+        <v/>
+      </c>
+      <c r="H6" s="15">
+        <f>H5/H3</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Backlog, years of current revenue</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="C7" s="17">
+        <f>Drivers!C6*1000/(Drivers!C10*4)</f>
+        <v/>
+      </c>
+      <c r="D7" s="17">
+        <f>Drivers!D6*1000/(Drivers!D10*4)</f>
+        <v/>
+      </c>
+      <c r="E7" s="17">
+        <f>Drivers!E6*1000/(Drivers!E10*4)</f>
+        <v/>
+      </c>
+      <c r="F7" s="17">
+        <f>Drivers!F6*1000/(Drivers!F10*4)</f>
+        <v/>
+      </c>
+      <c r="G7" s="17">
+        <f>Drivers!G6*1000/(Drivers!G10*4)</f>
+        <v/>
+      </c>
+      <c r="H7" s="17">
+        <f>Drivers!H6*1000/(Drivers!H10*4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Revenue per installed GPU-hour</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>USD/GPU-hour</t>
+        </is>
+      </c>
+      <c r="C8" s="17">
+        <f>Drivers!C10/Drivers!C9</f>
+        <v/>
+      </c>
+      <c r="D8" s="17">
+        <f>Drivers!D10/Drivers!D9</f>
+        <v/>
+      </c>
+      <c r="E8" s="17">
+        <f>Drivers!E10/Drivers!E9</f>
+        <v/>
+      </c>
+      <c r="F8" s="17">
+        <f>Drivers!F10/Drivers!F9</f>
+        <v/>
+      </c>
+      <c r="G8" s="17">
+        <f>Drivers!G10/Drivers!G9</f>
+        <v/>
+      </c>
+      <c r="H8" s="17">
+        <f>Drivers!H10/Drivers!H9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Cash cost per installed GPU-hour</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>USD/GPU-hour</t>
+        </is>
+      </c>
+      <c r="C9" s="17">
+        <f>(Drivers!C10-Drivers!C11)/Drivers!C9</f>
+        <v/>
+      </c>
+      <c r="D9" s="17">
+        <f>(Drivers!D10-Drivers!D11)/Drivers!D9</f>
+        <v/>
+      </c>
+      <c r="E9" s="17">
+        <f>(Drivers!E10-Drivers!E11)/Drivers!E9</f>
+        <v/>
+      </c>
+      <c r="F9" s="17">
+        <f>(Drivers!F10-Drivers!F11)/Drivers!F9</f>
+        <v/>
+      </c>
+      <c r="G9" s="17">
+        <f>(Drivers!G10-Drivers!G11)/Drivers!G9</f>
+        <v/>
+      </c>
+      <c r="H9" s="17">
+        <f>(Drivers!H10-Drivers!H11)/Drivers!H9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cash margin per installed GPU-hour</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>USD/GPU-hour</t>
+        </is>
+      </c>
+      <c r="C10" s="15">
+        <f>C8-C9</f>
+        <v/>
+      </c>
+      <c r="D10" s="15">
+        <f>D8-D9</f>
+        <v/>
+      </c>
+      <c r="E10" s="15">
+        <f>E8-E9</f>
+        <v/>
+      </c>
+      <c r="F10" s="15">
+        <f>F8-F9</f>
+        <v/>
+      </c>
+      <c r="G10" s="15">
+        <f>G8-G9</f>
+        <v/>
+      </c>
+      <c r="H10" s="15">
+        <f>H8-H9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Capital charge per installed GPU-hour</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>USD/GPU-hour</t>
+        </is>
+      </c>
+      <c r="C11" s="17">
+        <f>in_chip_cost*(1-in_residual_value_share/(1+in_financing_rate)^in_depreciation_years)*Drivers!C15/8760</f>
+        <v/>
+      </c>
+      <c r="D11" s="17">
+        <f>in_chip_cost*(1-in_residual_value_share/(1+in_financing_rate)^in_depreciation_years)*Drivers!D15/8760</f>
+        <v/>
+      </c>
+      <c r="E11" s="17">
+        <f>in_chip_cost*(1-in_residual_value_share/(1+in_financing_rate)^in_depreciation_years)*Drivers!E15/8760</f>
+        <v/>
+      </c>
+      <c r="F11" s="17">
+        <f>in_chip_cost*(1-in_residual_value_share/(1+in_financing_rate)^in_depreciation_years)*Drivers!F15/8760</f>
+        <v/>
+      </c>
+      <c r="G11" s="17">
+        <f>in_chip_cost*(1-in_residual_value_share/(1+in_financing_rate)^in_depreciation_years)*Drivers!G15/8760</f>
+        <v/>
+      </c>
+      <c r="H11" s="17">
+        <f>in_chip_cost*(1-in_residual_value_share/(1+in_financing_rate)^in_depreciation_years)*Drivers!H15/8760</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Fully loaded margin per installed GPU-hour</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>USD/GPU-hour</t>
+        </is>
+      </c>
+      <c r="C12" s="15">
+        <f>C10-C11</f>
+        <v/>
+      </c>
+      <c r="D12" s="15">
+        <f>D10-D11</f>
+        <v/>
+      </c>
+      <c r="E12" s="15">
+        <f>E10-E11</f>
+        <v/>
+      </c>
+      <c r="F12" s="15">
+        <f>F10-F11</f>
+        <v/>
+      </c>
+      <c r="G12" s="15">
+        <f>G10-G11</f>
+        <v/>
+      </c>
+      <c r="H12" s="15">
+        <f>H10-H11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Payback per GPU (engine)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="C13" s="17">
+        <f>IF(C10&gt;0,in_chip_cost/(C10*8760),"never")</f>
+        <v/>
+      </c>
+      <c r="D13" s="17">
+        <f>IF(D10&gt;0,in_chip_cost/(D10*8760),"never")</f>
+        <v/>
+      </c>
+      <c r="E13" s="17">
+        <f>IF(E10&gt;0,in_chip_cost/(E10*8760),"never")</f>
+        <v/>
+      </c>
+      <c r="F13" s="17">
+        <f>IF(F10&gt;0,in_chip_cost/(F10*8760),"never")</f>
+        <v/>
+      </c>
+      <c r="G13" s="17">
+        <f>IF(G10&gt;0,in_chip_cost/(G10*8760),"never")</f>
+        <v/>
+      </c>
+      <c r="H13" s="17">
+        <f>IF(H10&gt;0,in_chip_cost/(H10*8760),"never")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Payback, as disclosed by the company</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="C7" s="14">
+      <c r="C14" s="17">
         <f>in_disclosed_cash_payback_years</f>
         <v/>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Payback gap, model less disclosed</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="C8" s="15">
-        <f>C6-C7</f>
+      <c r="D14" s="17">
+        <f>in_disclosed_cash_payback_years</f>
+        <v/>
+      </c>
+      <c r="E14" s="17">
+        <f>in_disclosed_cash_payback_years</f>
+        <v/>
+      </c>
+      <c r="F14" s="17">
+        <f>in_disclosed_cash_payback_years</f>
+        <v/>
+      </c>
+      <c r="G14" s="17">
+        <f>in_disclosed_cash_payback_years</f>
+        <v/>
+      </c>
+      <c r="H14" s="17">
+        <f>in_disclosed_cash_payback_years</f>
         <v/>
       </c>
     </row>

</xml_diff>